<commit_message>
Diverge Azure demo CRM from AWS on two in-scope controls
The two demo CRMs were 39/41 identical designations, so the multi-tenant story
had no real per-scope split to show. Diverge two controls that ARE in scope and
assessed in the demo workbook so per-scope narratives genuinely differ:

- AU-6 (Audit Review): AWS=Shared, Azure=Customer (customer runs its own
  Sentinel workspace and owns review end-to-end on the Azure side).
- SC-13 (Crypto): AWS=Shared, Azure=Inherited (Azure Gov FIPS-validated Key
  Vault Managed HSM is fully inherited; no customer-side crypto).

Both are real, FedRAMP-plausible splits; the responsibility seam moves between
tenants, which is exactly what the boundary/per-scope narrative work assesses.
</commit_message>
<xml_diff>
--- a/demo/crm/Azure_Government_FedRAMP_High_CRM.xlsx
+++ b/demo/crm/Azure_Government_FedRAMP_High_CRM.xlsx
@@ -901,17 +901,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Microsoft reviews Azure-internal audit logs continuously via the Microsoft security operations team and reports relevant findings to customers per IR-6.</t>
+          <t>Microsoft provides the log sources (Activity Log, Entra audit, Defender for Cloud, Sentinel) but performs no review of customer-tenant audit records on the customer's behalf.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for reviewing customer Activity Logs, Defender for Cloud alerts, Microsoft Sentinel incidents, and application logs on the customer-defined cadence (minimum weekly for non-critical, continuous for critical). Reportable findings escalated per IR-6.</t>
+          <t>Customer is solely responsible for reviewing, analyzing, and reporting on customer Activity Logs, Defender for Cloud alerts, Microsoft Sentinel incidents, and application logs on the customer-defined cadence (minimum weekly for non-critical, continuous for critical). The customer operates the Sentinel workspace and escalates reportable findings per IR-6.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Inherited</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Microsoft provides FIPS 140-2 validated cryptographic modules within Azure Government via Key Vault, Managed HSM, and FIPS-validated service endpoints.</t>
+          <t>Microsoft provides FIPS 140-2 validated cryptographic modules within Azure Government via Key Vault, Managed HSM, and FIPS-validated service endpoints; the customer workload consumes only these validated modules and implements no independent cryptography.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Customer is responsible for using only FIPS 140-2 validated cryptographic implementations: enable FIPS-validated endpoints for customer service calls, configure FIPS mode in customer guest operating systems where supported, avoid non-FIPS algorithms in applications, and document customer cryptographic implementations in the SSP.</t>
+          <t>Customer fully inherits the FIPS 140-2 validated cryptographic modules provided by Azure Government. The customer SSP references the Azure Government FedRAMP High SSP as the authoritative source; no customer-side cryptographic implementation is required for this control.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">

</xml_diff>